<commit_message>
Latest tests.xlsm and code files
</commit_message>
<xml_diff>
--- a/docs/ExcelSteps_code_plan.xlsx
+++ b/docs/ExcelSteps_code_plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Mac\Home\Box Sync\Projects\Excel_Steps\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1EFBA31B-91E9-4EDA-9714-86EF31669448}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F9A23F9B-42B4-4902-81A6-D84480799AB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3225" yWindow="3600" windowWidth="28800" windowHeight="11588" xr2:uid="{C4957F84-F5CA-4AB5-8C48-0244E7B3E21C}"/>
+    <workbookView xWindow="1882" yWindow="1485" windowWidth="29888" windowHeight="14175" xr2:uid="{042F9CDB-90F3-4C2A-8CEA-B6980663A51E}"/>
   </bookViews>
   <sheets>
     <sheet name="ExcelSteps" sheetId="1" r:id="rId1"/>
@@ -554,7 +554,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6BB01DE-FE60-408E-AD4C-B18F52878B6C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1EEC2FD-5D1C-44AF-8350-107E62A66BA2}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:I28"/>
   <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1006,7 +1006,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C25" xr:uid="{88C97795-9214-42A9-8798-0591398E00A4}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C25" xr:uid="{E264F850-94D7-48EA-A95C-AF91A18E3DA9}">
       <formula1>"Col_Format,Col_Insert,Col_Delete,Col_Rename,Col_AddGroup,Col_CondFormat,Col_Dropdown,Tbl_FreezeRow1,Tbl_Sort,Tbl_SplitCols,Delete_FlagRows,Delete_RowsWithVal"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>